<commit_message>
make final semantic training runnable on Kaggle
</commit_message>
<xml_diff>
--- a/Bang_ke_hoach_SeqLogAD.xlsx
+++ b/Bang_ke_hoach_SeqLogAD.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive" sheetId="1" r:id="R1e08e2d1c99a4730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="Rab40ff8724614071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="3" r:id="Rd26e050d5c724817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="4" r:id="R89735ed6ee794e67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" r:id="R6066c9e3ce504e6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Sources" sheetId="6" r:id="Rf10f86214efa4ea9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Playbooks" sheetId="7" r:id="Rcb2aac62c2af404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive" sheetId="1" r:id="Rd87953879a9d4413"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="R8d6205396e8e4f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Register" sheetId="3" r:id="R0c766506b7ec44ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="4" r:id="R7f8a9fd14f2d43ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability" sheetId="5" r:id="R609d8ed961764def"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Sources" sheetId="6" r:id="Ra0a4278d09e14301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Playbooks" sheetId="7" r:id="R79ff99ba007045ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4943,7 +4943,7 @@
         <x:v>P2.PRE PASS before execution; independent adapter and scoring provenance, label-free source train/validation, semantic notebook and tests; REP-DG-001 conditional disposition recorded.</x:v>
       </x:c>
       <x:c r="K14" s="11" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="51.75" customHeight="1">
@@ -10358,7 +10358,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R670bf6f9ac714a25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4df33df8fd4ee5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11917,7 +11917,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77446562a0ea4a5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81363a3a3e0d48f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>